<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-18 18:58 UTC
</commit_message>
<xml_diff>
--- a/data/50001501 - EQ MIN LA HACIENDA B.xlsx
+++ b/data/50001501 - EQ MIN LA HACIENDA B.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2652" uniqueCount="434">
   <si>
     <t>50001501 - EQ. MIN. LA HACIENDA</t>
   </si>
@@ -5361,9 +5361,11 @@
       <c r="B62" s="5">
         <v>46073.76783866898</v>
       </c>
-      <c r="C62" s="6"/>
+      <c r="C62" s="5">
+        <v>46191.772903206016</v>
+      </c>
       <c r="D62" s="5">
-        <v>46150.78382966435</v>
+        <v>46191.77291996528</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>198</v>
@@ -5398,8 +5400,12 @@
       <c r="Q62" s="6"/>
       <c r="R62" s="6"/>
       <c r="S62" s="6"/>
-      <c r="T62" s="6"/>
-      <c r="U62" s="6"/>
+      <c r="T62" s="6">
+        <v>1</v>
+      </c>
+      <c r="U62" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-19 15:56 UTC
</commit_message>
<xml_diff>
--- a/data/50001501 - EQ MIN LA HACIENDA B.xlsx
+++ b/data/50001501 - EQ MIN LA HACIENDA B.xlsx
@@ -12334,7 +12334,7 @@
         <v>46191.796778240736</v>
       </c>
       <c r="D189" s="8">
-        <v>46191.79679478009</v>
+        <v>46192.64719054398</v>
       </c>
       <c r="E189" s="9" t="s">
         <v>373</v>
@@ -12395,9 +12395,11 @@
       <c r="B190" s="5">
         <v>46128.56718193287</v>
       </c>
-      <c r="C190" s="6"/>
+      <c r="C190" s="5">
+        <v>46192.64706778935</v>
+      </c>
       <c r="D190" s="5">
-        <v>46191.885307627315</v>
+        <v>46192.64706957176</v>
       </c>
       <c r="E190" s="6" t="s">
         <v>170</v>
@@ -12448,9 +12450,11 @@
       <c r="B191" s="8">
         <v>46128.567190092595</v>
       </c>
-      <c r="C191" s="9"/>
+      <c r="C191" s="8">
+        <v>46192.64718554398</v>
+      </c>
       <c r="D191" s="8">
-        <v>46191.88571938657</v>
+        <v>46192.647186875</v>
       </c>
       <c r="E191" s="9" t="s">
         <v>170</v>
@@ -13096,7 +13100,7 @@
       </c>
       <c r="C203" s="9"/>
       <c r="D203" s="8">
-        <v>46129.68352643518</v>
+        <v>46192.64707679398</v>
       </c>
       <c r="E203" s="9" t="s">
         <v>170</v>
@@ -13147,7 +13151,7 @@
       </c>
       <c r="C204" s="6"/>
       <c r="D204" s="5">
-        <v>46129.68352717593</v>
+        <v>46192.64719189815</v>
       </c>
       <c r="E204" s="6" t="s">
         <v>170</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-19 18:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001501 - EQ MIN LA HACIENDA B.xlsx
+++ b/data/50001501 - EQ MIN LA HACIENDA B.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2667" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2668" uniqueCount="436">
   <si>
     <t>50001501 - EQ. MIN. LA HACIENDA</t>
   </si>
@@ -520,6 +520,9 @@
     <t>OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2 ,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1214075676500814</t>
   </si>
   <si>
@@ -635,9 +638,6 @@
   </si>
   <si>
     <t>Preparación1 Materiales,Check Planos,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2,OT 4213 ZVN 1-9-86/2</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214075676500706</t>
@@ -4289,9 +4289,11 @@
       <c r="B42" s="5">
         <v>46073.76783873842</v>
       </c>
-      <c r="C42" s="6"/>
+      <c r="C42" s="5">
+        <v>46192.762426898145</v>
+      </c>
       <c r="D42" s="5">
-        <v>46142.64957708333</v>
+        <v>46192.76244386574</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>150</v>
@@ -4326,8 +4328,12 @@
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
       <c r="S42" s="6"/>
-      <c r="T42" s="6"/>
-      <c r="U42" s="6"/>
+      <c r="T42" s="6">
+        <v>1</v>
+      </c>
+      <c r="U42" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
@@ -4529,9 +4535,11 @@
       <c r="B46" s="5">
         <v>46090.493990891206</v>
       </c>
-      <c r="C46" s="6"/>
+      <c r="C46" s="5">
+        <v>46192.76206953704</v>
+      </c>
       <c r="D46" s="5">
-        <v>46129.678973692135</v>
+        <v>46192.76208826389</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>165</v>
@@ -4577,25 +4585,27 @@
         <v>31</v>
       </c>
       <c r="T46" s="6">
-        <v>0</v>
-      </c>
-      <c r="U46" s="10" t="s">
-        <v>106</v>
+        <v>1</v>
+      </c>
+      <c r="U46" s="12" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B47" s="8">
         <v>46128.56674524306</v>
       </c>
-      <c r="C47" s="9"/>
+      <c r="C47" s="8">
+        <v>46192.761913993054</v>
+      </c>
       <c r="D47" s="8">
-        <v>46191.79533020833</v>
+        <v>46192.7619153125</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>26</v>
@@ -4623,10 +4633,10 @@
         <v>165</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q47" s="9"/>
       <c r="R47" s="9"/>
@@ -4636,17 +4646,19 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B48" s="5">
         <v>46128.566755555556</v>
       </c>
-      <c r="C48" s="6"/>
+      <c r="C48" s="5">
+        <v>46192.76204381944</v>
+      </c>
       <c r="D48" s="5">
-        <v>46191.795324189814</v>
+        <v>46192.76205100694</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
@@ -4674,10 +4686,10 @@
         <v>165</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q48" s="6"/>
       <c r="R48" s="6"/>
@@ -4687,17 +4699,19 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B49" s="8">
         <v>46128.56676210648</v>
       </c>
-      <c r="C49" s="9"/>
+      <c r="C49" s="8">
+        <v>46192.76204465277</v>
+      </c>
       <c r="D49" s="8">
-        <v>46191.79531811342</v>
+        <v>46192.76205135416</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
@@ -4725,10 +4739,10 @@
         <v>165</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q49" s="9"/>
       <c r="R49" s="9"/>
@@ -4738,17 +4752,19 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B50" s="5">
         <v>46128.56676847222</v>
       </c>
-      <c r="C50" s="6"/>
+      <c r="C50" s="5">
+        <v>46192.76204524306</v>
+      </c>
       <c r="D50" s="5">
-        <v>46191.79531166666</v>
+        <v>46192.762051655096</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
@@ -4776,10 +4792,10 @@
         <v>165</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
@@ -4789,17 +4805,19 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B51" s="8">
         <v>46128.566774120365</v>
       </c>
-      <c r="C51" s="9"/>
+      <c r="C51" s="8">
+        <v>46192.76204579861</v>
+      </c>
       <c r="D51" s="8">
-        <v>46191.795306423606</v>
+        <v>46192.762051990736</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>26</v>
@@ -4827,10 +4845,10 @@
         <v>165</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q51" s="9"/>
       <c r="R51" s="9"/>
@@ -4840,17 +4858,19 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B52" s="5">
         <v>46128.566780127316</v>
       </c>
-      <c r="C52" s="6"/>
+      <c r="C52" s="5">
+        <v>46192.76204636574</v>
+      </c>
       <c r="D52" s="5">
-        <v>46191.7952890625</v>
+        <v>46192.76205229167</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
@@ -4878,10 +4898,10 @@
         <v>165</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4891,17 +4911,19 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B53" s="8">
         <v>46128.56678613426</v>
       </c>
-      <c r="C53" s="9"/>
+      <c r="C53" s="8">
+        <v>46192.76204696759</v>
+      </c>
       <c r="D53" s="8">
-        <v>46191.79528329861</v>
+        <v>46192.762052569444</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
@@ -4929,10 +4951,10 @@
         <v>165</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q53" s="9"/>
       <c r="R53" s="9"/>
@@ -4942,17 +4964,19 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B54" s="5">
         <v>46128.566790682875</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46192.7620475</v>
+      </c>
       <c r="D54" s="5">
-        <v>46191.79527969907</v>
+        <v>46192.7620528588</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
@@ -4980,10 +5004,10 @@
         <v>165</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
@@ -4993,17 +5017,19 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B55" s="8">
         <v>46128.5667968287</v>
       </c>
-      <c r="C55" s="9"/>
+      <c r="C55" s="8">
+        <v>46192.76204800926</v>
+      </c>
       <c r="D55" s="8">
-        <v>46191.795272557865</v>
+        <v>46192.76205314815</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
@@ -5031,10 +5057,10 @@
         <v>165</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P55" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q55" s="9"/>
       <c r="R55" s="9"/>
@@ -5044,17 +5070,19 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B56" s="5">
         <v>46128.56680166667</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46192.762048530094</v>
+      </c>
       <c r="D56" s="5">
-        <v>46191.795269375</v>
+        <v>46192.76205344907</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
@@ -5082,10 +5110,10 @@
         <v>165</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q56" s="6"/>
       <c r="R56" s="6"/>
@@ -5095,17 +5123,19 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B57" s="8">
         <v>46128.566807256946</v>
       </c>
-      <c r="C57" s="9"/>
+      <c r="C57" s="8">
+        <v>46192.76204903935</v>
+      </c>
       <c r="D57" s="8">
-        <v>46191.7952605787</v>
+        <v>46192.762053784725</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
@@ -5133,10 +5163,10 @@
         <v>165</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q57" s="9"/>
       <c r="R57" s="9"/>
@@ -5146,17 +5176,19 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B58" s="5">
         <v>46128.56681135416</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46192.76204957176</v>
+      </c>
       <c r="D58" s="5">
-        <v>46191.79525575231</v>
+        <v>46192.762054108796</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
@@ -5184,10 +5216,10 @@
         <v>165</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q58" s="6"/>
       <c r="R58" s="6"/>
@@ -5197,7 +5229,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B59" s="8">
         <v>46073.76783778935</v>
@@ -5209,7 +5241,7 @@
         <v>46097.81565780092</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>25</v>
@@ -5233,7 +5265,7 @@
         <v>26</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>26</v>
@@ -5250,7 +5282,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B60" s="5">
         <v>46073.767838078704</v>
@@ -5262,16 +5294,16 @@
         <v>46097.81529010416</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I60" s="5">
         <v>46041</v>
@@ -5289,13 +5321,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>147</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q60" s="5">
         <v>46041</v>
@@ -5315,7 +5347,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B61" s="8">
         <v>46073.7678383912</v>
@@ -5327,16 +5359,16 @@
         <v>46097.81562871528</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I61" s="8">
         <v>46043</v>
@@ -5354,13 +5386,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="P61" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q61" s="8">
         <v>46043</v>
@@ -5380,7 +5412,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B62" s="5">
         <v>46073.76783866898</v>
@@ -5392,7 +5424,7 @@
         <v>46191.77291996528</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>25</v>
@@ -5416,7 +5448,7 @@
         <v>26</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>26</v>
@@ -5433,7 +5465,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B63" s="8">
         <v>46073.767838935186</v>
@@ -5445,16 +5477,16 @@
         <v>46128.58222162037</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I63" s="8">
         <v>46045</v>
@@ -5472,13 +5504,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q63" s="8">
         <v>46045</v>
@@ -5498,7 +5530,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B64" s="5">
         <v>46073.76783921296</v>
@@ -5510,16 +5542,16 @@
         <v>46158.97116490741</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I64" s="5">
         <v>46050</v>
@@ -5537,13 +5569,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Q64" s="5">
         <v>46050</v>
@@ -5558,7 +5590,7 @@
         <v>1</v>
       </c>
       <c r="U64" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5575,16 +5607,16 @@
         <v>46129.68420498843</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I65" s="8">
         <v>46050</v>
@@ -5602,7 +5634,7 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O65" s="9" t="s">
         <v>210</v>
@@ -5630,16 +5662,16 @@
         <v>46129.684215497684</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I66" s="5">
         <v>46050</v>
@@ -5657,10 +5689,10 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>211</v>
@@ -5685,16 +5717,16 @@
         <v>46129.68427572917</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I67" s="8">
         <v>46050</v>
@@ -5712,10 +5744,10 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P67" s="9" t="s">
         <v>211</v>
@@ -5740,16 +5772,16 @@
         <v>46129.68422782407</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I68" s="5">
         <v>46050</v>
@@ -5767,10 +5799,10 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P68" s="6" t="s">
         <v>211</v>
@@ -5795,16 +5827,16 @@
         <v>46129.684293784725</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I69" s="8">
         <v>46050</v>
@@ -5822,10 +5854,10 @@
         <v>26</v>
       </c>
       <c r="N69" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P69" s="9" t="s">
         <v>211</v>
@@ -5850,16 +5882,16 @@
         <v>46129.68430454861</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I70" s="5">
         <v>46050</v>
@@ -5877,7 +5909,7 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>26</v>
@@ -5905,16 +5937,16 @@
         <v>46146.89516151621</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I71" s="8">
         <v>46050</v>
@@ -5932,7 +5964,7 @@
         <v>26</v>
       </c>
       <c r="N71" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O71" s="9" t="s">
         <v>218</v>
@@ -5960,16 +5992,16 @@
         <v>46146.89517496528</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I72" s="5">
         <v>46050</v>
@@ -5987,10 +6019,10 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>211</v>
@@ -6015,16 +6047,16 @@
         <v>46146.895229745365</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I73" s="8">
         <v>46050</v>
@@ -6042,10 +6074,10 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P73" s="9" t="s">
         <v>211</v>
@@ -6070,16 +6102,16 @@
         <v>46146.8951958449</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I74" s="5">
         <v>46050</v>
@@ -6097,10 +6129,10 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>211</v>
@@ -6125,16 +6157,16 @@
         <v>46146.8953142824</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I75" s="8">
         <v>46050</v>
@@ -6152,10 +6184,10 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P75" s="9" t="s">
         <v>211</v>
@@ -6180,16 +6212,16 @@
         <v>46146.895330486106</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I76" s="5">
         <v>46050</v>
@@ -6207,10 +6239,10 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>211</v>
@@ -6241,10 +6273,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I77" s="9"/>
       <c r="J77" s="8">
@@ -6260,13 +6292,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O77" s="9" t="s">
         <v>226</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Q77" s="8">
         <v>46055</v>
@@ -6298,16 +6330,16 @@
         <v>46129.6858422338</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="5">
@@ -6326,7 +6358,7 @@
         <v>225</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>228</v>
@@ -6351,16 +6383,16 @@
         <v>46129.68585466435</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I79" s="9"/>
       <c r="J79" s="8">
@@ -6379,7 +6411,7 @@
         <v>225</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P79" s="9" t="s">
         <v>228</v>
@@ -6404,16 +6436,16 @@
         <v>46129.68589648148</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I80" s="6"/>
       <c r="J80" s="5">
@@ -6432,7 +6464,7 @@
         <v>225</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>228</v>
@@ -6457,16 +6489,16 @@
         <v>46129.685910949076</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I81" s="9"/>
       <c r="J81" s="8">
@@ -6485,7 +6517,7 @@
         <v>225</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P81" s="9" t="s">
         <v>228</v>
@@ -6510,16 +6542,16 @@
         <v>46129.68592581019</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I82" s="6"/>
       <c r="J82" s="5">
@@ -6538,7 +6570,7 @@
         <v>225</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>228</v>
@@ -6563,16 +6595,16 @@
         <v>46129.68595777778</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I83" s="9"/>
       <c r="J83" s="8">
@@ -6591,7 +6623,7 @@
         <v>225</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P83" s="9" t="s">
         <v>228</v>
@@ -6616,16 +6648,16 @@
         <v>46146.897389502315</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I84" s="6"/>
       <c r="J84" s="5">
@@ -6644,7 +6676,7 @@
         <v>225</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>228</v>
@@ -6669,16 +6701,16 @@
         <v>46146.89739724537</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H85" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I85" s="9"/>
       <c r="J85" s="8">
@@ -6697,7 +6729,7 @@
         <v>225</v>
       </c>
       <c r="O85" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P85" s="9" t="s">
         <v>228</v>
@@ -6722,16 +6754,16 @@
         <v>46146.89740662037</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I86" s="6"/>
       <c r="J86" s="5">
@@ -6750,7 +6782,7 @@
         <v>225</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P86" s="6" t="s">
         <v>228</v>
@@ -6775,16 +6807,16 @@
         <v>46158.971886354164</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I87" s="9"/>
       <c r="J87" s="8">
@@ -6803,7 +6835,7 @@
         <v>225</v>
       </c>
       <c r="O87" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P87" s="9" t="s">
         <v>228</v>
@@ -6828,16 +6860,16 @@
         <v>46158.971913587964</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="5">
@@ -6856,7 +6888,7 @@
         <v>225</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P88" s="6" t="s">
         <v>228</v>
@@ -6881,16 +6913,16 @@
         <v>46158.971926909726</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I89" s="9"/>
       <c r="J89" s="8">
@@ -6909,7 +6941,7 @@
         <v>225</v>
       </c>
       <c r="O89" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P89" s="9" t="s">
         <v>228</v>
@@ -6934,7 +6966,7 @@
         <v>46191.79356716435</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>25</v>
@@ -6993,10 +7025,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I91" s="9"/>
       <c r="J91" s="8">
@@ -7012,13 +7044,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O91" s="9" t="s">
         <v>126</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q91" s="8">
         <v>46030</v>
@@ -7033,7 +7065,7 @@
         <v>0.2</v>
       </c>
       <c r="U91" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -7056,10 +7088,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I92" s="5">
         <v>46069</v>
@@ -7077,7 +7109,7 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O92" s="6" t="s">
         <v>117</v>
@@ -7121,10 +7153,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H93" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I93" s="9"/>
       <c r="J93" s="8">
@@ -7140,13 +7172,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O93" s="9" t="s">
         <v>108</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q93" s="8">
         <v>46014</v>
@@ -7161,7 +7193,7 @@
         <v>0</v>
       </c>
       <c r="U93" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
@@ -7184,10 +7216,10 @@
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I94" s="6"/>
       <c r="J94" s="5">
@@ -7203,7 +7235,7 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O94" s="6" t="s">
         <v>135</v>
@@ -7359,7 +7391,7 @@
         <v>46129.68866337963</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>26</v>
@@ -7389,7 +7421,7 @@
         <v>255</v>
       </c>
       <c r="O97" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P97" s="9" t="s">
         <v>258</v>
@@ -7414,7 +7446,7 @@
         <v>46129.688671157404</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7444,7 +7476,7 @@
         <v>255</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P98" s="6" t="s">
         <v>258</v>
@@ -7469,7 +7501,7 @@
         <v>46129.68868245371</v>
       </c>
       <c r="E99" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>26</v>
@@ -7499,7 +7531,7 @@
         <v>255</v>
       </c>
       <c r="O99" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P99" s="9" t="s">
         <v>258</v>
@@ -7524,7 +7556,7 @@
         <v>46129.688693171294</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
@@ -7554,7 +7586,7 @@
         <v>255</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P100" s="6" t="s">
         <v>258</v>
@@ -7579,7 +7611,7 @@
         <v>46129.68870375</v>
       </c>
       <c r="E101" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>26</v>
@@ -7609,7 +7641,7 @@
         <v>255</v>
       </c>
       <c r="O101" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P101" s="9" t="s">
         <v>258</v>
@@ -7634,7 +7666,7 @@
         <v>46158.974908738426</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
@@ -7664,7 +7696,7 @@
         <v>255</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P102" s="6" t="s">
         <v>258</v>
@@ -7689,7 +7721,7 @@
         <v>46158.97511034722</v>
       </c>
       <c r="E103" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>26</v>
@@ -7719,7 +7751,7 @@
         <v>255</v>
       </c>
       <c r="O103" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P103" s="9" t="s">
         <v>258</v>
@@ -7744,7 +7776,7 @@
         <v>46158.975184641204</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
@@ -7774,7 +7806,7 @@
         <v>255</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P104" s="6" t="s">
         <v>258</v>
@@ -7799,7 +7831,7 @@
         <v>46191.79465511574</v>
       </c>
       <c r="E105" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>26</v>
@@ -7829,7 +7861,7 @@
         <v>255</v>
       </c>
       <c r="O105" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P105" s="9" t="s">
         <v>258</v>
@@ -7854,7 +7886,7 @@
         <v>46191.79466190972</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -7884,7 +7916,7 @@
         <v>255</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P106" s="6" t="s">
         <v>258</v>
@@ -7909,7 +7941,7 @@
         <v>46191.79466734953</v>
       </c>
       <c r="E107" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>26</v>
@@ -7939,7 +7971,7 @@
         <v>255</v>
       </c>
       <c r="O107" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P107" s="9" t="s">
         <v>258</v>
@@ -7964,7 +7996,7 @@
         <v>46191.79473116898</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
@@ -7994,7 +8026,7 @@
         <v>255</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P108" s="6" t="s">
         <v>258</v>
@@ -8082,7 +8114,7 @@
         <v>46157.498779988426</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>26</v>
@@ -8110,7 +8142,7 @@
         <v>271</v>
       </c>
       <c r="O110" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P110" s="6" t="s">
         <v>273</v>
@@ -8135,7 +8167,7 @@
         <v>46157.49878368055</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>26</v>
@@ -8163,7 +8195,7 @@
         <v>271</v>
       </c>
       <c r="O111" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P111" s="9" t="s">
         <v>273</v>
@@ -8188,7 +8220,7 @@
         <v>46157.498788240744</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8216,7 +8248,7 @@
         <v>271</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P112" s="6" t="s">
         <v>273</v>
@@ -8241,7 +8273,7 @@
         <v>46157.49879474537</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>26</v>
@@ -8269,7 +8301,7 @@
         <v>271</v>
       </c>
       <c r="O113" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P113" s="9" t="s">
         <v>273</v>
@@ -8294,7 +8326,7 @@
         <v>46157.49884443287</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>26</v>
@@ -8322,7 +8354,7 @@
         <v>271</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P114" s="6" t="s">
         <v>273</v>
@@ -8347,7 +8379,7 @@
         <v>46158.97491230324</v>
       </c>
       <c r="E115" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>26</v>
@@ -8375,7 +8407,7 @@
         <v>271</v>
       </c>
       <c r="O115" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P115" s="9" t="s">
         <v>273</v>
@@ -8400,7 +8432,7 @@
         <v>46158.975114155095</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8428,7 +8460,7 @@
         <v>271</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P116" s="6" t="s">
         <v>273</v>
@@ -8453,7 +8485,7 @@
         <v>46158.97518857638</v>
       </c>
       <c r="E117" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>26</v>
@@ -8481,7 +8513,7 @@
         <v>271</v>
       </c>
       <c r="O117" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P117" s="9" t="s">
         <v>273</v>
@@ -8506,7 +8538,7 @@
         <v>46191.794660555555</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
@@ -8534,7 +8566,7 @@
         <v>271</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P118" s="6" t="s">
         <v>273</v>
@@ -8559,7 +8591,7 @@
         <v>46191.79466525463</v>
       </c>
       <c r="E119" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>26</v>
@@ -8587,7 +8619,7 @@
         <v>271</v>
       </c>
       <c r="O119" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P119" s="9" t="s">
         <v>273</v>
@@ -8612,7 +8644,7 @@
         <v>46191.794671875</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>26</v>
@@ -8640,7 +8672,7 @@
         <v>271</v>
       </c>
       <c r="O120" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P120" s="6" t="s">
         <v>273</v>
@@ -8665,7 +8697,7 @@
         <v>46191.79473787037</v>
       </c>
       <c r="E121" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>26</v>
@@ -8693,7 +8725,7 @@
         <v>271</v>
       </c>
       <c r="O121" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P121" s="9" t="s">
         <v>273</v>
@@ -8783,7 +8815,7 @@
         <v>46157.49878587963</v>
       </c>
       <c r="E123" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>26</v>
@@ -8813,7 +8845,7 @@
         <v>286</v>
       </c>
       <c r="O123" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P123" s="9" t="s">
         <v>288</v>
@@ -8838,7 +8870,7 @@
         <v>46157.49878896991</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
@@ -8868,7 +8900,7 @@
         <v>286</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P124" s="6" t="s">
         <v>288</v>
@@ -8893,7 +8925,7 @@
         <v>46157.49879293982</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>26</v>
@@ -8923,7 +8955,7 @@
         <v>286</v>
       </c>
       <c r="O125" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P125" s="9" t="s">
         <v>288</v>
@@ -8948,7 +8980,7 @@
         <v>46157.498799560184</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>26</v>
@@ -8978,7 +9010,7 @@
         <v>286</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P126" s="6" t="s">
         <v>288</v>
@@ -9003,7 +9035,7 @@
         <v>46157.49885005787</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>26</v>
@@ -9033,7 +9065,7 @@
         <v>286</v>
       </c>
       <c r="O127" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P127" s="9" t="s">
         <v>288</v>
@@ -9058,7 +9090,7 @@
         <v>46157.4988055787</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
@@ -9088,7 +9120,7 @@
         <v>286</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P128" s="6" t="s">
         <v>288</v>
@@ -9113,7 +9145,7 @@
         <v>46157.49893354166</v>
       </c>
       <c r="E129" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>26</v>
@@ -9143,7 +9175,7 @@
         <v>286</v>
       </c>
       <c r="O129" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P129" s="9" t="s">
         <v>288</v>
@@ -9168,7 +9200,7 @@
         <v>46157.49900008102</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F130" s="6" t="s">
         <v>26</v>
@@ -9198,7 +9230,7 @@
         <v>286</v>
       </c>
       <c r="O130" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P130" s="6" t="s">
         <v>288</v>
@@ -9223,7 +9255,7 @@
         <v>46191.7937930787</v>
       </c>
       <c r="E131" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>26</v>
@@ -9253,7 +9285,7 @@
         <v>286</v>
       </c>
       <c r="O131" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P131" s="9" t="s">
         <v>288</v>
@@ -9278,7 +9310,7 @@
         <v>46191.79424862268</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>26</v>
@@ -9308,7 +9340,7 @@
         <v>286</v>
       </c>
       <c r="O132" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P132" s="6" t="s">
         <v>288</v>
@@ -9333,7 +9365,7 @@
         <v>46191.79439909723</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>26</v>
@@ -9363,7 +9395,7 @@
         <v>286</v>
       </c>
       <c r="O133" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P133" s="9" t="s">
         <v>288</v>
@@ -9388,7 +9420,7 @@
         <v>46191.79452946759</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>26</v>
@@ -9418,7 +9450,7 @@
         <v>286</v>
       </c>
       <c r="O134" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P134" s="6" t="s">
         <v>288</v>
@@ -9506,7 +9538,7 @@
         <v>46157.49801296296</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F136" s="6" t="s">
         <v>26</v>
@@ -9536,7 +9568,7 @@
         <v>301</v>
       </c>
       <c r="O136" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P136" s="6" t="s">
         <v>304</v>
@@ -9561,7 +9593,7 @@
         <v>46157.49802616898</v>
       </c>
       <c r="E137" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>26</v>
@@ -9591,7 +9623,7 @@
         <v>301</v>
       </c>
       <c r="O137" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P137" s="9" t="s">
         <v>304</v>
@@ -9616,7 +9648,7 @@
         <v>46157.49803459491</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F138" s="6" t="s">
         <v>26</v>
@@ -9646,7 +9678,7 @@
         <v>301</v>
       </c>
       <c r="O138" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P138" s="6" t="s">
         <v>304</v>
@@ -9671,7 +9703,7 @@
         <v>46157.4980403588</v>
       </c>
       <c r="E139" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>26</v>
@@ -9701,7 +9733,7 @@
         <v>301</v>
       </c>
       <c r="O139" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P139" s="9" t="s">
         <v>304</v>
@@ -9726,7 +9758,7 @@
         <v>46157.49804547454</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F140" s="6" t="s">
         <v>26</v>
@@ -9756,7 +9788,7 @@
         <v>301</v>
       </c>
       <c r="O140" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P140" s="6" t="s">
         <v>304</v>
@@ -9781,7 +9813,7 @@
         <v>46157.49809685185</v>
       </c>
       <c r="E141" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>26</v>
@@ -9811,7 +9843,7 @@
         <v>301</v>
       </c>
       <c r="O141" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P141" s="9" t="s">
         <v>304</v>
@@ -9836,7 +9868,7 @@
         <v>46157.498176423614</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F142" s="6" t="s">
         <v>26</v>
@@ -9866,7 +9898,7 @@
         <v>301</v>
       </c>
       <c r="O142" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P142" s="6" t="s">
         <v>304</v>
@@ -9891,7 +9923,7 @@
         <v>46157.49829290509</v>
       </c>
       <c r="E143" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>26</v>
@@ -9921,7 +9953,7 @@
         <v>301</v>
       </c>
       <c r="O143" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P143" s="9" t="s">
         <v>304</v>
@@ -9946,7 +9978,7 @@
         <v>46191.793351631946</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F144" s="6" t="s">
         <v>26</v>
@@ -9976,7 +10008,7 @@
         <v>301</v>
       </c>
       <c r="O144" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P144" s="6" t="s">
         <v>304</v>
@@ -10001,7 +10033,7 @@
         <v>46191.79344340278</v>
       </c>
       <c r="E145" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>26</v>
@@ -10031,7 +10063,7 @@
         <v>301</v>
       </c>
       <c r="O145" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P145" s="9" t="s">
         <v>304</v>
@@ -10056,7 +10088,7 @@
         <v>46191.79351224537</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F146" s="6" t="s">
         <v>26</v>
@@ -10086,7 +10118,7 @@
         <v>301</v>
       </c>
       <c r="O146" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P146" s="6" t="s">
         <v>304</v>
@@ -10111,7 +10143,7 @@
         <v>46191.7935915625</v>
       </c>
       <c r="E147" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>26</v>
@@ -10141,7 +10173,7 @@
         <v>301</v>
       </c>
       <c r="O147" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P147" s="9" t="s">
         <v>304</v>
@@ -10212,7 +10244,7 @@
         <v>1</v>
       </c>
       <c r="U148" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.25">
@@ -10229,7 +10261,7 @@
         <v>46191.79532310185</v>
       </c>
       <c r="E149" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>26</v>
@@ -10257,7 +10289,7 @@
         <v>317</v>
       </c>
       <c r="O149" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P149" s="9" t="s">
         <v>319</v>
@@ -10282,7 +10314,7 @@
         <v>46191.7953178125</v>
       </c>
       <c r="E150" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F150" s="6" t="s">
         <v>26</v>
@@ -10310,7 +10342,7 @@
         <v>317</v>
       </c>
       <c r="O150" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P150" s="6" t="s">
         <v>319</v>
@@ -10335,7 +10367,7 @@
         <v>46191.79531292824</v>
       </c>
       <c r="E151" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>26</v>
@@ -10363,7 +10395,7 @@
         <v>317</v>
       </c>
       <c r="O151" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P151" s="9" t="s">
         <v>319</v>
@@ -10388,7 +10420,7 @@
         <v>46191.79530751157</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F152" s="6" t="s">
         <v>26</v>
@@ -10416,7 +10448,7 @@
         <v>317</v>
       </c>
       <c r="O152" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P152" s="6" t="s">
         <v>323</v>
@@ -10441,7 +10473,7 @@
         <v>46191.79530002315</v>
       </c>
       <c r="E153" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>26</v>
@@ -10469,7 +10501,7 @@
         <v>317</v>
       </c>
       <c r="O153" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P153" s="9" t="s">
         <v>319</v>
@@ -10494,7 +10526,7 @@
         <v>46191.79528344907</v>
       </c>
       <c r="E154" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F154" s="6" t="s">
         <v>26</v>
@@ -10522,7 +10554,7 @@
         <v>317</v>
       </c>
       <c r="O154" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P154" s="6" t="s">
         <v>319</v>
@@ -10547,7 +10579,7 @@
         <v>46191.79527836805</v>
       </c>
       <c r="E155" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>26</v>
@@ -10575,7 +10607,7 @@
         <v>317</v>
       </c>
       <c r="O155" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P155" s="9" t="s">
         <v>319</v>
@@ -10600,7 +10632,7 @@
         <v>46191.79527357639</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F156" s="6" t="s">
         <v>26</v>
@@ -10628,7 +10660,7 @@
         <v>317</v>
       </c>
       <c r="O156" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P156" s="6" t="s">
         <v>319</v>
@@ -10653,7 +10685,7 @@
         <v>46191.795267951384</v>
       </c>
       <c r="E157" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>26</v>
@@ -10681,7 +10713,7 @@
         <v>317</v>
       </c>
       <c r="O157" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P157" s="9" t="s">
         <v>319</v>
@@ -10706,7 +10738,7 @@
         <v>46191.79526363426</v>
       </c>
       <c r="E158" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F158" s="6" t="s">
         <v>26</v>
@@ -10734,7 +10766,7 @@
         <v>317</v>
       </c>
       <c r="O158" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P158" s="6" t="s">
         <v>319</v>
@@ -10759,7 +10791,7 @@
         <v>46191.79525519676</v>
       </c>
       <c r="E159" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>26</v>
@@ -10787,7 +10819,7 @@
         <v>317</v>
       </c>
       <c r="O159" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P159" s="9" t="s">
         <v>319</v>
@@ -10812,7 +10844,7 @@
         <v>46191.795250173614</v>
       </c>
       <c r="E160" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F160" s="6" t="s">
         <v>26</v>
@@ -10840,7 +10872,7 @@
         <v>317</v>
       </c>
       <c r="O160" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P160" s="6" t="s">
         <v>319</v>
@@ -10911,7 +10943,7 @@
         <v>1</v>
       </c>
       <c r="U161" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="162" spans="1:21" x14ac:dyDescent="0.25">
@@ -10925,10 +10957,10 @@
         <v>46191.79662097222</v>
       </c>
       <c r="D162" s="5">
-        <v>46191.796622511574</v>
+        <v>46192.76192157407</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F162" s="6" t="s">
         <v>26</v>
@@ -10956,7 +10988,7 @@
         <v>333</v>
       </c>
       <c r="O162" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P162" s="6" t="s">
         <v>336</v>
@@ -10978,10 +11010,10 @@
         <v>46191.796464733794</v>
       </c>
       <c r="D163" s="8">
-        <v>46191.796466134256</v>
+        <v>46192.76206450231</v>
       </c>
       <c r="E163" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>26</v>
@@ -11009,7 +11041,7 @@
         <v>333</v>
       </c>
       <c r="O163" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P163" s="9" t="s">
         <v>336</v>
@@ -11031,10 +11063,10 @@
         <v>46191.79639053241</v>
       </c>
       <c r="D164" s="5">
-        <v>46191.79639206019</v>
+        <v>46192.76206446759</v>
       </c>
       <c r="E164" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F164" s="6" t="s">
         <v>26</v>
@@ -11062,7 +11094,7 @@
         <v>333</v>
       </c>
       <c r="O164" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P164" s="6" t="s">
         <v>336</v>
@@ -11084,10 +11116,10 @@
         <v>46191.79629663195</v>
       </c>
       <c r="D165" s="8">
-        <v>46191.796298194444</v>
+        <v>46192.76206489583</v>
       </c>
       <c r="E165" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>26</v>
@@ -11115,7 +11147,7 @@
         <v>333</v>
       </c>
       <c r="O165" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P165" s="9" t="s">
         <v>336</v>
@@ -11137,10 +11169,10 @@
         <v>46191.79617204861</v>
       </c>
       <c r="D166" s="5">
-        <v>46191.79617392361</v>
+        <v>46192.76206432871</v>
       </c>
       <c r="E166" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F166" s="6" t="s">
         <v>26</v>
@@ -11168,7 +11200,7 @@
         <v>333</v>
       </c>
       <c r="O166" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P166" s="6" t="s">
         <v>336</v>
@@ -11190,10 +11222,10 @@
         <v>46191.79610912037</v>
       </c>
       <c r="D167" s="8">
-        <v>46191.796110972224</v>
+        <v>46192.76206412037</v>
       </c>
       <c r="E167" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>26</v>
@@ -11221,7 +11253,7 @@
         <v>333</v>
       </c>
       <c r="O167" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P167" s="9" t="s">
         <v>336</v>
@@ -11243,10 +11275,10 @@
         <v>46191.796043587965</v>
       </c>
       <c r="D168" s="5">
-        <v>46191.7960453125</v>
+        <v>46192.762064131944</v>
       </c>
       <c r="E168" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F168" s="6" t="s">
         <v>26</v>
@@ -11274,7 +11306,7 @@
         <v>333</v>
       </c>
       <c r="O168" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P168" s="6" t="s">
         <v>336</v>
@@ -11296,10 +11328,10 @@
         <v>46191.795971342595</v>
       </c>
       <c r="D169" s="8">
-        <v>46191.79597306713</v>
+        <v>46192.762064131944</v>
       </c>
       <c r="E169" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>26</v>
@@ -11327,7 +11359,7 @@
         <v>333</v>
       </c>
       <c r="O169" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P169" s="9" t="s">
         <v>336</v>
@@ -11349,10 +11381,10 @@
         <v>46191.79585572917</v>
       </c>
       <c r="D170" s="5">
-        <v>46191.79585737269</v>
+        <v>46192.76206414352</v>
       </c>
       <c r="E170" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F170" s="6" t="s">
         <v>26</v>
@@ -11380,7 +11412,7 @@
         <v>333</v>
       </c>
       <c r="O170" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P170" s="6" t="s">
         <v>336</v>
@@ -11402,10 +11434,10 @@
         <v>46191.795773958336</v>
       </c>
       <c r="D171" s="8">
-        <v>46191.79577540509</v>
+        <v>46192.76206392361</v>
       </c>
       <c r="E171" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>26</v>
@@ -11433,7 +11465,7 @@
         <v>333</v>
       </c>
       <c r="O171" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P171" s="9" t="s">
         <v>336</v>
@@ -11455,10 +11487,10 @@
         <v>46191.79563440972</v>
       </c>
       <c r="D172" s="5">
-        <v>46191.795636319446</v>
+        <v>46192.76206421296</v>
       </c>
       <c r="E172" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F172" s="6" t="s">
         <v>26</v>
@@ -11486,7 +11518,7 @@
         <v>333</v>
       </c>
       <c r="O172" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P172" s="6" t="s">
         <v>336</v>
@@ -11508,10 +11540,10 @@
         <v>46191.79554900463</v>
       </c>
       <c r="D173" s="8">
-        <v>46191.79555090278</v>
+        <v>46192.762064305556</v>
       </c>
       <c r="E173" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>26</v>
@@ -11539,7 +11571,7 @@
         <v>333</v>
       </c>
       <c r="O173" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P173" s="9" t="s">
         <v>336</v>
@@ -11672,7 +11704,7 @@
         <v>46191.885297430556</v>
       </c>
       <c r="E176" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F176" s="6" t="s">
         <v>26</v>
@@ -11700,7 +11732,7 @@
         <v>352</v>
       </c>
       <c r="O176" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P176" s="6" t="s">
         <v>357</v>
@@ -11723,7 +11755,7 @@
         <v>46191.88571055555</v>
       </c>
       <c r="E177" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>26</v>
@@ -11751,7 +11783,7 @@
         <v>352</v>
       </c>
       <c r="O177" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P177" s="9" t="s">
         <v>357</v>
@@ -11774,7 +11806,7 @@
         <v>46191.88526354167</v>
       </c>
       <c r="E178" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F178" s="6" t="s">
         <v>26</v>
@@ -11802,7 +11834,7 @@
         <v>352</v>
       </c>
       <c r="O178" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P178" s="6" t="s">
         <v>357</v>
@@ -11825,7 +11857,7 @@
         <v>46191.88525847222</v>
       </c>
       <c r="E179" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>26</v>
@@ -11853,7 +11885,7 @@
         <v>352</v>
       </c>
       <c r="O179" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P179" s="9" t="s">
         <v>357</v>
@@ -11876,7 +11908,7 @@
         <v>46191.88525349537</v>
       </c>
       <c r="E180" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F180" s="6" t="s">
         <v>26</v>
@@ -11904,7 +11936,7 @@
         <v>352</v>
       </c>
       <c r="O180" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P180" s="6" t="s">
         <v>357</v>
@@ -11927,7 +11959,7 @@
         <v>46191.885310405094</v>
       </c>
       <c r="E181" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>26</v>
@@ -11955,7 +11987,7 @@
         <v>352</v>
       </c>
       <c r="O181" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P181" s="9" t="s">
         <v>357</v>
@@ -11978,7 +12010,7 @@
         <v>46191.796051701385</v>
       </c>
       <c r="E182" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F182" s="6" t="s">
         <v>26</v>
@@ -12006,7 +12038,7 @@
         <v>352</v>
       </c>
       <c r="O182" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P182" s="6" t="s">
         <v>357</v>
@@ -12029,7 +12061,7 @@
         <v>46191.795977581016</v>
       </c>
       <c r="E183" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>26</v>
@@ -12057,7 +12089,7 @@
         <v>352</v>
       </c>
       <c r="O183" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P183" s="9" t="s">
         <v>365</v>
@@ -12080,7 +12112,7 @@
         <v>46191.795861736115</v>
       </c>
       <c r="E184" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F184" s="6" t="s">
         <v>26</v>
@@ -12108,7 +12140,7 @@
         <v>352</v>
       </c>
       <c r="O184" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P184" s="6" t="s">
         <v>357</v>
@@ -12131,7 +12163,7 @@
         <v>46191.795781168985</v>
       </c>
       <c r="E185" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>26</v>
@@ -12159,7 +12191,7 @@
         <v>352</v>
       </c>
       <c r="O185" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P185" s="9" t="s">
         <v>357</v>
@@ -12182,7 +12214,7 @@
         <v>46191.795643460646</v>
       </c>
       <c r="E186" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F186" s="6" t="s">
         <v>26</v>
@@ -12210,7 +12242,7 @@
         <v>352</v>
       </c>
       <c r="O186" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P186" s="6" t="s">
         <v>357</v>
@@ -12233,7 +12265,7 @@
         <v>46191.795556990735</v>
       </c>
       <c r="E187" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>26</v>
@@ -12261,7 +12293,7 @@
         <v>352</v>
       </c>
       <c r="O187" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P187" s="9" t="s">
         <v>357</v>
@@ -12402,7 +12434,7 @@
         <v>46192.64706957176</v>
       </c>
       <c r="E190" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F190" s="6" t="s">
         <v>26</v>
@@ -12432,7 +12464,7 @@
         <v>373</v>
       </c>
       <c r="O190" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P190" s="6" t="s">
         <v>375</v>
@@ -12457,7 +12489,7 @@
         <v>46192.647186875</v>
       </c>
       <c r="E191" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>26</v>
@@ -12487,7 +12519,7 @@
         <v>373</v>
       </c>
       <c r="O191" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P191" s="9" t="s">
         <v>375</v>
@@ -12510,7 +12542,7 @@
         <v>46191.8852687037</v>
       </c>
       <c r="E192" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F192" s="6" t="s">
         <v>26</v>
@@ -12540,7 +12572,7 @@
         <v>373</v>
       </c>
       <c r="O192" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P192" s="6" t="s">
         <v>375</v>
@@ -12563,7 +12595,7 @@
         <v>46191.88526256944</v>
       </c>
       <c r="E193" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>26</v>
@@ -12593,7 +12625,7 @@
         <v>373</v>
       </c>
       <c r="O193" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P193" s="9" t="s">
         <v>375</v>
@@ -12616,7 +12648,7 @@
         <v>46191.885259710645</v>
       </c>
       <c r="E194" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F194" s="6" t="s">
         <v>26</v>
@@ -12646,7 +12678,7 @@
         <v>373</v>
       </c>
       <c r="O194" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P194" s="6" t="s">
         <v>375</v>
@@ -12669,7 +12701,7 @@
         <v>46191.88531537037</v>
       </c>
       <c r="E195" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>26</v>
@@ -12699,7 +12731,7 @@
         <v>373</v>
       </c>
       <c r="O195" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P195" s="9" t="s">
         <v>375</v>
@@ -12722,7 +12754,7 @@
         <v>46129.68320027778</v>
       </c>
       <c r="E196" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F196" s="6" t="s">
         <v>26</v>
@@ -12752,7 +12784,7 @@
         <v>373</v>
       </c>
       <c r="O196" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P196" s="6" t="s">
         <v>375</v>
@@ -12775,7 +12807,7 @@
         <v>46129.68320100695</v>
       </c>
       <c r="E197" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>26</v>
@@ -12805,7 +12837,7 @@
         <v>373</v>
       </c>
       <c r="O197" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P197" s="9" t="s">
         <v>375</v>
@@ -12828,7 +12860,7 @@
         <v>46129.683201747685</v>
       </c>
       <c r="E198" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F198" s="6" t="s">
         <v>26</v>
@@ -12858,7 +12890,7 @@
         <v>373</v>
       </c>
       <c r="O198" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P198" s="6" t="s">
         <v>26</v>
@@ -12881,7 +12913,7 @@
         <v>46129.683202500004</v>
       </c>
       <c r="E199" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>26</v>
@@ -12911,7 +12943,7 @@
         <v>373</v>
       </c>
       <c r="O199" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P199" s="9" t="s">
         <v>375</v>
@@ -12934,7 +12966,7 @@
         <v>46129.683203252316</v>
       </c>
       <c r="E200" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F200" s="6" t="s">
         <v>26</v>
@@ -12964,7 +12996,7 @@
         <v>373</v>
       </c>
       <c r="O200" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P200" s="6" t="s">
         <v>375</v>
@@ -12987,7 +13019,7 @@
         <v>46129.683203981476</v>
       </c>
       <c r="E201" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>26</v>
@@ -13017,7 +13049,7 @@
         <v>373</v>
       </c>
       <c r="O201" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P201" s="9" t="s">
         <v>375</v>
@@ -13048,10 +13080,10 @@
         <v>26</v>
       </c>
       <c r="G202" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H202" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I202" s="6"/>
       <c r="J202" s="5">
@@ -13103,16 +13135,16 @@
         <v>46192.64707679398</v>
       </c>
       <c r="E203" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G203" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H203" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I203" s="9"/>
       <c r="J203" s="8">
@@ -13131,7 +13163,7 @@
         <v>388</v>
       </c>
       <c r="O203" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P203" s="9" t="s">
         <v>390</v>
@@ -13154,16 +13186,16 @@
         <v>46192.64719189815</v>
       </c>
       <c r="E204" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F204" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G204" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H204" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I204" s="6"/>
       <c r="J204" s="5">
@@ -13182,7 +13214,7 @@
         <v>388</v>
       </c>
       <c r="O204" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P204" s="6" t="s">
         <v>390</v>
@@ -13205,16 +13237,16 @@
         <v>46129.68352791667</v>
       </c>
       <c r="E205" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G205" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H205" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I205" s="9"/>
       <c r="J205" s="8">
@@ -13233,7 +13265,7 @@
         <v>388</v>
       </c>
       <c r="O205" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P205" s="9" t="s">
         <v>390</v>
@@ -13256,16 +13288,16 @@
         <v>46129.683528657406</v>
       </c>
       <c r="E206" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F206" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G206" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H206" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I206" s="6"/>
       <c r="J206" s="5">
@@ -13284,7 +13316,7 @@
         <v>388</v>
       </c>
       <c r="O206" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P206" s="6" t="s">
         <v>390</v>
@@ -13307,16 +13339,16 @@
         <v>46129.68352943287</v>
       </c>
       <c r="E207" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G207" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H207" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I207" s="9"/>
       <c r="J207" s="8">
@@ -13335,7 +13367,7 @@
         <v>388</v>
       </c>
       <c r="O207" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P207" s="9" t="s">
         <v>390</v>
@@ -13358,16 +13390,16 @@
         <v>46129.68353019676</v>
       </c>
       <c r="E208" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F208" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G208" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H208" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I208" s="6"/>
       <c r="J208" s="5">
@@ -13386,7 +13418,7 @@
         <v>388</v>
       </c>
       <c r="O208" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P208" s="6" t="s">
         <v>390</v>
@@ -13409,16 +13441,16 @@
         <v>46129.683530891205</v>
       </c>
       <c r="E209" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G209" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H209" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I209" s="9"/>
       <c r="J209" s="8">
@@ -13437,7 +13469,7 @@
         <v>388</v>
       </c>
       <c r="O209" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P209" s="9" t="s">
         <v>397</v>
@@ -13460,16 +13492,16 @@
         <v>46129.68353159723</v>
       </c>
       <c r="E210" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F210" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G210" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H210" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I210" s="6"/>
       <c r="J210" s="5">
@@ -13488,7 +13520,7 @@
         <v>388</v>
       </c>
       <c r="O210" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P210" s="6" t="s">
         <v>397</v>
@@ -13511,16 +13543,16 @@
         <v>46129.68353232639</v>
       </c>
       <c r="E211" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G211" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H211" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I211" s="9"/>
       <c r="J211" s="8">
@@ -13539,7 +13571,7 @@
         <v>388</v>
       </c>
       <c r="O211" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P211" s="9" t="s">
         <v>397</v>
@@ -13562,16 +13594,16 @@
         <v>46129.683533125004</v>
       </c>
       <c r="E212" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F212" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G212" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H212" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I212" s="6"/>
       <c r="J212" s="5">
@@ -13590,7 +13622,7 @@
         <v>388</v>
       </c>
       <c r="O212" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P212" s="6" t="s">
         <v>397</v>
@@ -13613,16 +13645,16 @@
         <v>46129.68353385417</v>
       </c>
       <c r="E213" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G213" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H213" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I213" s="9"/>
       <c r="J213" s="8">
@@ -13641,7 +13673,7 @@
         <v>388</v>
       </c>
       <c r="O213" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P213" s="9" t="s">
         <v>397</v>
@@ -13664,16 +13696,16 @@
         <v>46129.68353459491</v>
       </c>
       <c r="E214" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F214" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G214" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H214" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I214" s="6"/>
       <c r="J214" s="5">
@@ -13692,7 +13724,7 @@
         <v>388</v>
       </c>
       <c r="O214" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P214" s="6" t="s">
         <v>397</v>
@@ -13723,10 +13755,10 @@
         <v>26</v>
       </c>
       <c r="G215" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H215" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I215" s="9"/>
       <c r="J215" s="8">
@@ -13778,16 +13810,16 @@
         <v>46129.69451681713</v>
       </c>
       <c r="E216" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F216" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G216" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H216" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I216" s="6"/>
       <c r="J216" s="5">
@@ -13806,7 +13838,7 @@
         <v>404</v>
       </c>
       <c r="O216" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P216" s="6" t="s">
         <v>404</v>
@@ -13829,16 +13861,16 @@
         <v>46129.69454358796</v>
       </c>
       <c r="E217" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G217" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H217" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I217" s="9"/>
       <c r="J217" s="8">
@@ -13857,7 +13889,7 @@
         <v>404</v>
       </c>
       <c r="O217" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P217" s="9" t="s">
         <v>404</v>
@@ -13880,16 +13912,16 @@
         <v>46129.694564502315</v>
       </c>
       <c r="E218" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F218" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G218" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H218" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I218" s="6"/>
       <c r="J218" s="5">
@@ -13908,7 +13940,7 @@
         <v>404</v>
       </c>
       <c r="O218" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P218" s="6" t="s">
         <v>404</v>
@@ -13931,16 +13963,16 @@
         <v>46129.694584282406</v>
       </c>
       <c r="E219" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G219" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H219" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I219" s="9"/>
       <c r="J219" s="8">
@@ -13959,7 +13991,7 @@
         <v>404</v>
       </c>
       <c r="O219" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P219" s="9" t="s">
         <v>404</v>
@@ -13982,16 +14014,16 @@
         <v>46129.69460693287</v>
       </c>
       <c r="E220" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F220" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G220" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H220" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I220" s="6"/>
       <c r="J220" s="5">
@@ -14010,7 +14042,7 @@
         <v>404</v>
       </c>
       <c r="O220" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P220" s="6" t="s">
         <v>404</v>
@@ -14033,16 +14065,16 @@
         <v>46129.69462627315</v>
       </c>
       <c r="E221" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G221" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H221" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I221" s="9"/>
       <c r="J221" s="8">
@@ -14061,7 +14093,7 @@
         <v>404</v>
       </c>
       <c r="O221" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P221" s="9" t="s">
         <v>404</v>
@@ -14084,16 +14116,16 @@
         <v>46129.69465064815</v>
       </c>
       <c r="E222" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F222" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G222" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H222" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I222" s="6"/>
       <c r="J222" s="5">
@@ -14112,7 +14144,7 @@
         <v>404</v>
       </c>
       <c r="O222" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P222" s="6" t="s">
         <v>404</v>
@@ -14135,16 +14167,16 @@
         <v>46129.69467157408</v>
       </c>
       <c r="E223" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G223" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H223" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I223" s="9"/>
       <c r="J223" s="8">
@@ -14163,7 +14195,7 @@
         <v>404</v>
       </c>
       <c r="O223" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P223" s="9" t="s">
         <v>404</v>
@@ -14186,16 +14218,16 @@
         <v>46129.69469225695</v>
       </c>
       <c r="E224" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F224" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G224" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H224" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I224" s="6"/>
       <c r="J224" s="5">
@@ -14214,7 +14246,7 @@
         <v>404</v>
       </c>
       <c r="O224" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P224" s="6" t="s">
         <v>404</v>
@@ -14237,16 +14269,16 @@
         <v>46129.694713379635</v>
       </c>
       <c r="E225" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G225" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H225" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I225" s="9"/>
       <c r="J225" s="8">
@@ -14265,7 +14297,7 @@
         <v>404</v>
       </c>
       <c r="O225" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P225" s="9" t="s">
         <v>404</v>
@@ -14288,16 +14320,16 @@
         <v>46129.694735682875</v>
       </c>
       <c r="E226" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F226" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G226" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H226" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I226" s="6"/>
       <c r="J226" s="5">
@@ -14316,7 +14348,7 @@
         <v>404</v>
       </c>
       <c r="O226" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P226" s="6" t="s">
         <v>404</v>
@@ -14339,16 +14371,16 @@
         <v>46129.694774895834</v>
       </c>
       <c r="E227" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G227" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H227" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I227" s="9"/>
       <c r="J227" s="8">
@@ -14367,7 +14399,7 @@
         <v>404</v>
       </c>
       <c r="O227" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P227" s="9" t="s">
         <v>404</v>
@@ -14485,7 +14517,7 @@
         <v>0</v>
       </c>
       <c r="U229" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="230" spans="1:21" x14ac:dyDescent="0.25">
@@ -14548,7 +14580,7 @@
         <v>0</v>
       </c>
       <c r="U230" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="231" spans="1:21" x14ac:dyDescent="0.25">
@@ -14660,7 +14692,7 @@
         <v>0</v>
       </c>
       <c r="U232" s="12" t="s">
-        <v>208</v>
+        <v>169</v>
       </c>
     </row>
     <row r="233" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-21 17:05 UTC
</commit_message>
<xml_diff>
--- a/data/50001501 - EQ MIN LA HACIENDA B.xlsx
+++ b/data/50001501 - EQ MIN LA HACIENDA B.xlsx
@@ -11646,7 +11646,7 @@
         <v>46193.56105240741</v>
       </c>
       <c r="D175" s="8">
-        <v>46193.56105853009</v>
+        <v>46194.709360277775</v>
       </c>
       <c r="E175" s="9" t="s">
         <v>352</v>
@@ -11696,8 +11696,8 @@
       <c r="T175" s="9">
         <v>1</v>
       </c>
-      <c r="U175" s="11" t="s">
-        <v>32</v>
+      <c r="U175" s="12" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="176" spans="1:21" x14ac:dyDescent="0.25">
@@ -11707,9 +11707,11 @@
       <c r="B176" s="5">
         <v>46128.56704659722</v>
       </c>
-      <c r="C176" s="6"/>
+      <c r="C176" s="5">
+        <v>46194.70201375</v>
+      </c>
       <c r="D176" s="5">
-        <v>46191.885297430556</v>
+        <v>46194.70208606482</v>
       </c>
       <c r="E176" s="6" t="s">
         <v>171</v>
@@ -11758,9 +11760,11 @@
       <c r="B177" s="8">
         <v>46128.56705305555</v>
       </c>
-      <c r="C177" s="9"/>
+      <c r="C177" s="8">
+        <v>46194.70201552083</v>
+      </c>
       <c r="D177" s="8">
-        <v>46191.88571055555</v>
+        <v>46194.70208699074</v>
       </c>
       <c r="E177" s="9" t="s">
         <v>171</v>
@@ -11809,9 +11813,11 @@
       <c r="B178" s="5">
         <v>46128.567060127316</v>
       </c>
-      <c r="C178" s="6"/>
+      <c r="C178" s="5">
+        <v>46194.702016446754</v>
+      </c>
       <c r="D178" s="5">
-        <v>46191.88526354167</v>
+        <v>46194.702087638885</v>
       </c>
       <c r="E178" s="6" t="s">
         <v>171</v>
@@ -11860,9 +11866,11 @@
       <c r="B179" s="8">
         <v>46128.56706601851</v>
       </c>
-      <c r="C179" s="9"/>
+      <c r="C179" s="8">
+        <v>46194.702017372685</v>
+      </c>
       <c r="D179" s="8">
-        <v>46191.88525847222</v>
+        <v>46194.70208831019</v>
       </c>
       <c r="E179" s="9" t="s">
         <v>171</v>
@@ -11911,9 +11919,11 @@
       <c r="B180" s="5">
         <v>46128.56707302084</v>
       </c>
-      <c r="C180" s="6"/>
+      <c r="C180" s="5">
+        <v>46194.70201841435</v>
+      </c>
       <c r="D180" s="5">
-        <v>46191.88525349537</v>
+        <v>46194.70208899306</v>
       </c>
       <c r="E180" s="6" t="s">
         <v>171</v>
@@ -11962,9 +11972,11 @@
       <c r="B181" s="8">
         <v>46128.56708030093</v>
       </c>
-      <c r="C181" s="9"/>
+      <c r="C181" s="8">
+        <v>46194.702019247685</v>
+      </c>
       <c r="D181" s="8">
-        <v>46191.885310405094</v>
+        <v>46194.70208959491</v>
       </c>
       <c r="E181" s="9" t="s">
         <v>171</v>
@@ -12013,9 +12025,11 @@
       <c r="B182" s="5">
         <v>46128.56708731482</v>
       </c>
-      <c r="C182" s="6"/>
+      <c r="C182" s="5">
+        <v>46194.70206814815</v>
+      </c>
       <c r="D182" s="5">
-        <v>46191.796051701385</v>
+        <v>46194.70209015046</v>
       </c>
       <c r="E182" s="6" t="s">
         <v>171</v>
@@ -12064,9 +12078,11 @@
       <c r="B183" s="8">
         <v>46128.567094432874</v>
       </c>
-      <c r="C183" s="9"/>
+      <c r="C183" s="8">
+        <v>46194.70207223379</v>
+      </c>
       <c r="D183" s="8">
-        <v>46191.795977581016</v>
+        <v>46194.702090729166</v>
       </c>
       <c r="E183" s="9" t="s">
         <v>171</v>
@@ -12115,9 +12131,11 @@
       <c r="B184" s="5">
         <v>46128.56710209491</v>
       </c>
-      <c r="C184" s="6"/>
+      <c r="C184" s="5">
+        <v>46194.70207326389</v>
+      </c>
       <c r="D184" s="5">
-        <v>46191.795861736115</v>
+        <v>46194.702091354164</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>171</v>
@@ -12166,9 +12184,11 @@
       <c r="B185" s="8">
         <v>46128.56710883102</v>
       </c>
-      <c r="C185" s="9"/>
+      <c r="C185" s="8">
+        <v>46194.70207423611</v>
+      </c>
       <c r="D185" s="8">
-        <v>46191.795781168985</v>
+        <v>46194.70209196759</v>
       </c>
       <c r="E185" s="9" t="s">
         <v>171</v>
@@ -12217,9 +12237,11 @@
       <c r="B186" s="5">
         <v>46128.56711633102</v>
       </c>
-      <c r="C186" s="6"/>
+      <c r="C186" s="5">
+        <v>46194.70208087963</v>
+      </c>
       <c r="D186" s="5">
-        <v>46191.795643460646</v>
+        <v>46194.7020958912</v>
       </c>
       <c r="E186" s="6" t="s">
         <v>171</v>
@@ -12268,9 +12290,11 @@
       <c r="B187" s="8">
         <v>46128.56712334491</v>
       </c>
-      <c r="C187" s="9"/>
+      <c r="C187" s="8">
+        <v>46194.70208171297</v>
+      </c>
       <c r="D187" s="8">
-        <v>46191.795556990735</v>
+        <v>46194.70209655093</v>
       </c>
       <c r="E187" s="9" t="s">
         <v>171</v>
@@ -12319,9 +12343,11 @@
       <c r="B188" s="5">
         <v>46191.895071886574</v>
       </c>
-      <c r="C188" s="6"/>
+      <c r="C188" s="5">
+        <v>46194.702082511576</v>
+      </c>
       <c r="D188" s="5">
-        <v>46191.895473171295</v>
+        <v>46194.702097546295</v>
       </c>
       <c r="E188" s="6" t="s">
         <v>371</v>
@@ -12374,7 +12400,7 @@
         <v>46191.796778240736</v>
       </c>
       <c r="D189" s="8">
-        <v>46192.64719054398</v>
+        <v>46194.70536553241</v>
       </c>
       <c r="E189" s="9" t="s">
         <v>373</v>
@@ -12439,7 +12465,7 @@
         <v>46192.64706778935</v>
       </c>
       <c r="D190" s="5">
-        <v>46192.64706957176</v>
+        <v>46194.70885945602</v>
       </c>
       <c r="E190" s="6" t="s">
         <v>171</v>
@@ -12494,7 +12520,7 @@
         <v>46192.64718554398</v>
       </c>
       <c r="D191" s="8">
-        <v>46192.647186875</v>
+        <v>46194.706768668984</v>
       </c>
       <c r="E191" s="9" t="s">
         <v>171</v>
@@ -12547,7 +12573,7 @@
       </c>
       <c r="C192" s="6"/>
       <c r="D192" s="5">
-        <v>46191.8852687037</v>
+        <v>46194.70287113426</v>
       </c>
       <c r="E192" s="6" t="s">
         <v>171</v>
@@ -12600,7 +12626,7 @@
       </c>
       <c r="C193" s="9"/>
       <c r="D193" s="8">
-        <v>46191.88526256944</v>
+        <v>46194.70272818287</v>
       </c>
       <c r="E193" s="9" t="s">
         <v>171</v>
@@ -12653,7 +12679,7 @@
       </c>
       <c r="C194" s="6"/>
       <c r="D194" s="5">
-        <v>46191.885259710645</v>
+        <v>46194.70217247686</v>
       </c>
       <c r="E194" s="6" t="s">
         <v>171</v>
@@ -12706,7 +12732,7 @@
       </c>
       <c r="C195" s="9"/>
       <c r="D195" s="8">
-        <v>46191.88531537037</v>
+        <v>46194.70884659722</v>
       </c>
       <c r="E195" s="9" t="s">
         <v>171</v>
@@ -12759,7 +12785,7 @@
       </c>
       <c r="C196" s="6"/>
       <c r="D196" s="5">
-        <v>46129.68320027778</v>
+        <v>46194.7024039699</v>
       </c>
       <c r="E196" s="6" t="s">
         <v>171</v>
@@ -12812,7 +12838,7 @@
       </c>
       <c r="C197" s="9"/>
       <c r="D197" s="8">
-        <v>46129.68320100695</v>
+        <v>46194.70536497685</v>
       </c>
       <c r="E197" s="9" t="s">
         <v>171</v>
@@ -12865,7 +12891,7 @@
       </c>
       <c r="C198" s="6"/>
       <c r="D198" s="5">
-        <v>46129.683201747685</v>
+        <v>46194.70870311343</v>
       </c>
       <c r="E198" s="6" t="s">
         <v>171</v>
@@ -12918,7 +12944,7 @@
       </c>
       <c r="C199" s="9"/>
       <c r="D199" s="8">
-        <v>46129.683202500004</v>
+        <v>46194.70256980324</v>
       </c>
       <c r="E199" s="9" t="s">
         <v>171</v>
@@ -12971,7 +12997,7 @@
       </c>
       <c r="C200" s="6"/>
       <c r="D200" s="5">
-        <v>46129.683203252316</v>
+        <v>46194.70497310185</v>
       </c>
       <c r="E200" s="6" t="s">
         <v>171</v>
@@ -13024,7 +13050,7 @@
       </c>
       <c r="C201" s="9"/>
       <c r="D201" s="8">
-        <v>46129.683203981476</v>
+        <v>46194.703054178244</v>
       </c>
       <c r="E201" s="9" t="s">
         <v>171</v>
@@ -13497,7 +13523,7 @@
       </c>
       <c r="C210" s="6"/>
       <c r="D210" s="5">
-        <v>46129.68353159723</v>
+        <v>46194.70536717593</v>
       </c>
       <c r="E210" s="6" t="s">
         <v>171</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 01:17 UTC
</commit_message>
<xml_diff>
--- a/data/50001501 - EQ MIN LA HACIENDA B.xlsx
+++ b/data/50001501 - EQ MIN LA HACIENDA B.xlsx
@@ -12400,7 +12400,7 @@
         <v>46191.796778240736</v>
       </c>
       <c r="D189" s="8">
-        <v>46194.70536553241</v>
+        <v>46194.7453605787</v>
       </c>
       <c r="E189" s="9" t="s">
         <v>373</v>
@@ -12450,8 +12450,8 @@
       <c r="T189" s="9">
         <v>1</v>
       </c>
-      <c r="U189" s="11" t="s">
-        <v>32</v>
+      <c r="U189" s="12" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="190" spans="1:21" x14ac:dyDescent="0.25">
@@ -12571,9 +12571,11 @@
       <c r="B192" s="5">
         <v>46128.567196550925</v>
       </c>
-      <c r="C192" s="6"/>
+      <c r="C192" s="5">
+        <v>46194.745200694444</v>
+      </c>
       <c r="D192" s="5">
-        <v>46194.70287113426</v>
+        <v>46194.7452021412</v>
       </c>
       <c r="E192" s="6" t="s">
         <v>171</v>
@@ -12624,9 +12626,11 @@
       <c r="B193" s="8">
         <v>46128.56720474537</v>
       </c>
-      <c r="C193" s="9"/>
+      <c r="C193" s="8">
+        <v>46194.7452541088</v>
+      </c>
       <c r="D193" s="8">
-        <v>46194.70272818287</v>
+        <v>46194.74525607639</v>
       </c>
       <c r="E193" s="9" t="s">
         <v>171</v>
@@ -12677,9 +12681,11 @@
       <c r="B194" s="5">
         <v>46128.56721146991</v>
       </c>
-      <c r="C194" s="6"/>
+      <c r="C194" s="5">
+        <v>46194.74508903935</v>
+      </c>
       <c r="D194" s="5">
-        <v>46194.70217247686</v>
+        <v>46194.74509084491</v>
       </c>
       <c r="E194" s="6" t="s">
         <v>171</v>
@@ -12730,9 +12736,11 @@
       <c r="B195" s="8">
         <v>46128.56721795139</v>
       </c>
-      <c r="C195" s="9"/>
+      <c r="C195" s="8">
+        <v>46194.74486503472</v>
+      </c>
       <c r="D195" s="8">
-        <v>46194.70884659722</v>
+        <v>46194.74486726851</v>
       </c>
       <c r="E195" s="9" t="s">
         <v>171</v>
@@ -12783,9 +12791,11 @@
       <c r="B196" s="5">
         <v>46128.56722548611</v>
       </c>
-      <c r="C196" s="6"/>
+      <c r="C196" s="5">
+        <v>46194.74534504629</v>
+      </c>
       <c r="D196" s="5">
-        <v>46194.7024039699</v>
+        <v>46194.74534685185</v>
       </c>
       <c r="E196" s="6" t="s">
         <v>171</v>
@@ -12836,9 +12846,11 @@
       <c r="B197" s="8">
         <v>46128.567233333335</v>
       </c>
-      <c r="C197" s="9"/>
+      <c r="C197" s="8">
+        <v>46194.7449961574</v>
+      </c>
       <c r="D197" s="8">
-        <v>46194.70536497685</v>
+        <v>46194.74499798611</v>
       </c>
       <c r="E197" s="9" t="s">
         <v>171</v>
@@ -12889,9 +12901,11 @@
       <c r="B198" s="5">
         <v>46128.56724010417</v>
       </c>
-      <c r="C198" s="6"/>
+      <c r="C198" s="5">
+        <v>46194.744955497685</v>
+      </c>
       <c r="D198" s="5">
-        <v>46194.70870311343</v>
+        <v>46194.74495716435</v>
       </c>
       <c r="E198" s="6" t="s">
         <v>171</v>
@@ -12942,9 +12956,11 @@
       <c r="B199" s="8">
         <v>46128.56724606482</v>
       </c>
-      <c r="C199" s="9"/>
+      <c r="C199" s="8">
+        <v>46194.74529594908</v>
+      </c>
       <c r="D199" s="8">
-        <v>46194.70256980324</v>
+        <v>46194.74529774305</v>
       </c>
       <c r="E199" s="9" t="s">
         <v>171</v>
@@ -12995,9 +13011,11 @@
       <c r="B200" s="5">
         <v>46128.56725237268</v>
       </c>
-      <c r="C200" s="6"/>
+      <c r="C200" s="5">
+        <v>46194.745028819445</v>
+      </c>
       <c r="D200" s="5">
-        <v>46194.70497310185</v>
+        <v>46194.74503064815</v>
       </c>
       <c r="E200" s="6" t="s">
         <v>171</v>
@@ -13048,9 +13066,11 @@
       <c r="B201" s="8">
         <v>46128.56725944445</v>
       </c>
-      <c r="C201" s="9"/>
+      <c r="C201" s="8">
+        <v>46194.745127002316</v>
+      </c>
       <c r="D201" s="8">
-        <v>46194.703054178244</v>
+        <v>46194.74512893519</v>
       </c>
       <c r="E201" s="9" t="s">
         <v>171</v>
@@ -13268,7 +13288,7 @@
       </c>
       <c r="C205" s="9"/>
       <c r="D205" s="8">
-        <v>46129.68352791667</v>
+        <v>46194.745209120374</v>
       </c>
       <c r="E205" s="9" t="s">
         <v>171</v>
@@ -13319,7 +13339,7 @@
       </c>
       <c r="C206" s="6"/>
       <c r="D206" s="5">
-        <v>46129.683528657406</v>
+        <v>46194.74526217593</v>
       </c>
       <c r="E206" s="6" t="s">
         <v>171</v>
@@ -13370,7 +13390,7 @@
       </c>
       <c r="C207" s="9"/>
       <c r="D207" s="8">
-        <v>46129.68352943287</v>
+        <v>46194.74509618056</v>
       </c>
       <c r="E207" s="9" t="s">
         <v>171</v>
@@ -13421,7 +13441,7 @@
       </c>
       <c r="C208" s="6"/>
       <c r="D208" s="5">
-        <v>46129.68353019676</v>
+        <v>46194.74487355324</v>
       </c>
       <c r="E208" s="6" t="s">
         <v>171</v>
@@ -13472,7 +13492,7 @@
       </c>
       <c r="C209" s="9"/>
       <c r="D209" s="8">
-        <v>46129.683530891205</v>
+        <v>46194.74535369213</v>
       </c>
       <c r="E209" s="9" t="s">
         <v>171</v>
@@ -13574,7 +13594,7 @@
       </c>
       <c r="C211" s="9"/>
       <c r="D211" s="8">
-        <v>46129.68353232639</v>
+        <v>46194.74500435185</v>
       </c>
       <c r="E211" s="9" t="s">
         <v>171</v>
@@ -13625,7 +13645,7 @@
       </c>
       <c r="C212" s="6"/>
       <c r="D212" s="5">
-        <v>46129.683533125004</v>
+        <v>46194.74530193287</v>
       </c>
       <c r="E212" s="6" t="s">
         <v>171</v>
@@ -13676,7 +13696,7 @@
       </c>
       <c r="C213" s="9"/>
       <c r="D213" s="8">
-        <v>46129.68353385417</v>
+        <v>46194.7450368287</v>
       </c>
       <c r="E213" s="9" t="s">
         <v>171</v>
@@ -13727,7 +13747,7 @@
       </c>
       <c r="C214" s="6"/>
       <c r="D214" s="5">
-        <v>46129.68353459491</v>
+        <v>46194.74513560185</v>
       </c>
       <c r="E214" s="6" t="s">
         <v>171</v>

</xml_diff>